<commit_message>
Update: 2026-07-12 07:59 SAST
</commit_message>
<xml_diff>
--- a/exports/Brewfather_Batches_Summary.xlsx
+++ b/exports/Brewfather_Batches_Summary.xlsx
@@ -758,7 +758,9 @@
       <c r="M2" s="3" t="n">
         <v>1.016</v>
       </c>
-      <c r="N2" s="3" t="n"/>
+      <c r="N2" s="3" t="n">
+        <v>1.016</v>
+      </c>
       <c r="O2" s="4" t="n">
         <v>5.38</v>
       </c>
@@ -808,7 +810,9 @@
       <c r="AE2" s="4" t="n">
         <v>10</v>
       </c>
-      <c r="AF2" s="4" t="n"/>
+      <c r="AF2" s="4" t="n">
+        <v>10</v>
+      </c>
       <c r="AG2" s="4" t="n">
         <v>59.6</v>
       </c>

</xml_diff>

<commit_message>
Update: 2026-08-02 05:24 SAST
</commit_message>
<xml_diff>
--- a/exports/Brewfather_Batches_Summary.xlsx
+++ b/exports/Brewfather_Batches_Summary.xlsx
@@ -756,11 +756,11 @@
         <v>1.048</v>
       </c>
       <c r="M2" s="3" t="n">
-        <v>1.01</v>
+        <v>1.009</v>
       </c>
       <c r="N2" s="3" t="n"/>
       <c r="O2" s="4" t="n">
-        <v>4.99</v>
+        <v>5.12</v>
       </c>
       <c r="P2" s="4" t="n">
         <v>5</v>

</xml_diff>